<commit_message>
Complete Day 32 Cash Flow Intelligence and Capital Allocation Report
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -945,7 +945,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -989,11 +989,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
-      </c>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1043,7 +1039,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1091,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1143,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1195,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1247,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1299,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1351,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1403,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1456,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Distress Signal</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1508,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1560,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1612,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1664,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1716,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1769,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1825,7 +1821,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1873,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1925,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1977,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2029,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2081,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2133,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2185,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2237,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -2293,7 +2289,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2341,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2397,7 +2393,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2445,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2497,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2549,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2602,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2654,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2707,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2759,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2811,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2863,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Unknown</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2915,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2967,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Pre-Revenue</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3019,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3072,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3124,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3176,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3229,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3281,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3337,7 +3333,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Unknown</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3385,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3437,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3494,7 +3490,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3546,7 +3542,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3594,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3646,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3698,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3755,7 +3751,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3803,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3855,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3907,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3959,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4012,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4064,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4116,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4168,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4220,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4272,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4324,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4376,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4429,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4481,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4533,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4589,7 +4585,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4638,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4690,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4742,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4798,7 +4794,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -4850,7 +4846,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4903,7 +4899,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4952,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5004,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5056,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -5113,7 +5109,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -5165,7 +5161,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5213,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>Deleveraging</t>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5265,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>Distress</t>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>

</xml_diff>